<commit_message>
aportes a configuracion de datos
</commit_message>
<xml_diff>
--- a/Color/LogicDocs/formulas y funciones .xlsx
+++ b/Color/LogicDocs/formulas y funciones .xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://coatsplc-my.sharepoint.com/personal/elkinduvan_quebradaguapacha_coats_com/Documents/Escritorio/Colorimetria/Color/LogicDocs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1060" documentId="8_{9F78D261-5971-4E36-A791-098E2ABB119D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{505A8C73-BF1A-4B90-8D3A-1129F6B1D33A}"/>
+  <xr:revisionPtr revIDLastSave="1132" documentId="8_{9F78D261-5971-4E36-A791-098E2ABB119D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5A586577-7C02-4391-B8F9-780D0F2601CF}"/>
   <bookViews>
-    <workbookView xWindow="10695" yWindow="0" windowWidth="11010" windowHeight="12885" xr2:uid="{74F1A0B1-3ED8-4C59-B930-9B261CE40F5C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" firstSheet="1" activeTab="3" xr2:uid="{74F1A0B1-3ED8-4C59-B930-9B261CE40F5C}"/>
   </bookViews>
   <sheets>
     <sheet name="CALCULO SAMPLE COMPARISON " sheetId="3" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="140">
   <si>
     <t>CMC(2.1)</t>
   </si>
@@ -377,18 +377,9 @@
     <t>b</t>
   </si>
   <si>
-    <t>variacion</t>
-  </si>
-  <si>
     <t>(((ll-ls)/ls)*100)</t>
   </si>
   <si>
-    <t>l</t>
-  </si>
-  <si>
-    <t>((std- lot)/std)</t>
-  </si>
-  <si>
     <t xml:space="preserve">dl </t>
   </si>
   <si>
@@ -396,6 +387,190 @@
   </si>
   <si>
     <t>dh</t>
+  </si>
+  <si>
+    <t>varacion</t>
+  </si>
+  <si>
+    <t>Valor Abs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L </t>
+  </si>
+  <si>
+    <t>lot-std</t>
+  </si>
+  <si>
+    <t>(std-lot)/std</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">_      </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Si esta opaco y si esta oscuro; entonces </t>
+    </r>
+  </si>
+  <si>
+    <t>(-)</t>
+  </si>
+  <si>
+    <t>(=) restar brillante 0%</t>
+  </si>
+  <si>
+    <t>Receta # 1</t>
+  </si>
+  <si>
+    <t>Receta # 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Receta # 3 </t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">_  </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Si esta opaco y si esta oscuro; entonces </t>
+    </r>
+  </si>
+  <si>
+    <t>(=) restar oscuro 0%</t>
+  </si>
+  <si>
+    <t>_+%</t>
+  </si>
+  <si>
+    <t>------</t>
+  </si>
+  <si>
+    <t>-------</t>
+  </si>
+  <si>
+    <t>oscuro (-)</t>
+  </si>
+  <si>
+    <t>✔</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">_  </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Si esta brillante y si esta claro; </t>
+    </r>
+  </si>
+  <si>
+    <t>(+)</t>
+  </si>
+  <si>
+    <t>(=) sumar opaco 0%</t>
+  </si>
+  <si>
+    <t>--------</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Si esta opaco y si esta esta claro; entonces </t>
+    </r>
+  </si>
+  <si>
+    <t>(=) sumar brillante 0%</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>claro (+)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">brillante </t>
+  </si>
+  <si>
+    <t xml:space="preserve">opaco </t>
+  </si>
+  <si>
+    <t>delta %</t>
+  </si>
+  <si>
+    <t>La teoría de Kubelka-Munk (1931) es un modelo matemático fundamental que describe cómo la luz interactúa con materiales difusores y absorbentes, como pinturas, recubrimientos o polvos, relacionando la reflectancia con el coeficiente de absorción (\(K\)) y dispersión (\(S\)). Se basa en dos flujos de luz (uno ascendente y otro descendente) para predecir color, opacidad y concentración de pigmentos.Aspectos Clave de la Ley de Kubelka-MunkFundamento: Desarrollada por Paul Kubelka y Franz Munk, simplifica la transferencia radiativa asumiendo que la luz se difunde en medios espesos.Ecuación Fundamental: Para una muestra de espesor infinito o muy grueso, la reflectancia se relaciona con \(K\) (absorción) y \(S\) (dispersión) mediante:\(\frac{K}{S}=\frac{(1-R_{\infty })^{2}}{2R_{\infty }}\)Donde \(R_{\infty }\) es la reflectancia de una capa gruesa (reflectancia absoluta).Aplicaciones Principales:Ciencia del Color: Predecir el color y la opacidad de pinturas y recubrimientos.Espectroscopia (DRIFTS): Analizar muestras sólidas, donde se usa para convertir la reflectancia difusa en una señal linealmente proporcional a la concentración del analito.Caracterización de Materiales: Determinar la banda prohibida (band gap) de semiconductores en polvo.Modelo de Dos Flujos: Considera un flujo de luz hacia abajo (incidente) y otro hacia arriba (dispersado) para modelar la dispersión y la absorción.Limitaciones: Funciona mejor en medios turbios y con alta difusión. No se aplica con precisión en películas muy delgadas o materiales transparentes.</t>
+  </si>
+  <si>
+    <t>UTILIZACION DE TEORIA EN EL PROGRAMA</t>
+  </si>
+  <si>
+    <t>El Salto de "Espacio Color" a "Fuerza de Color" (K/S)
+El programa no calcula sobre los valores $L^*, a^*, b^*$ directamente. Utiliza la ley de Kubelka-Munk.
+•	El Problema: El color no es lineal. Si duplicas la cantidad de colorante en una tina, el hilo no se ve "el doble de oscuro".
+•	La Solución Dinámica: El programa convierte la reflectancia en una función llamada $K/S$ (Absorción/Dispersión). Esto permite que el $\Delta\%$ que ves en pantalla sea directamente proporcional a la masa de colorante.
+•	Resultado: Si el programa dice $-2.60\%$, es porque calculó cuánta energía de luz se está perdiendo y cuántos gramos de colorante real compensan esa pérdida.
+2. Ponderación Multiluminante (Metamerismo)
+Un cálculo dinámico significa que el programa está analizando el lote bajo tres realidades distintas simultáneamente (D65, TL84, A).
+•	Si el lote se desvía mucho bajo luz de tungsteno (A) pero poco bajo luz de día (D65), el programa no te da un promedio simple.
+•	Dinámica: El algoritmo prioriza el iluminante principal de Coats, pero ajusta la recomendación de receta para que el color sea estable en todas las luces. El Excel, al ser estático, solo ve un escenario a la vez.
+3. El Algoritmo de Diferencia de Color (CMC 2:1 o CIE2000)
+•	Cálculo Dinámico (Programa): Crea un elipsoide de tolerancia. Si el color es un amarillo brillante, el elipsoide se expande (somos menos sensibles). Si el color es un neutro, el elipsoide se encoge.
+•	Por eso el programa puede decir que un lote "CUMPLE" aunque numéricamente parezca desviado, o viceversa.
+Resumen del Proceso Interno
+Cada vez que presionas "Iniciar Escaneo", ocurre esta secuencia en milisegundos:
+1.	Normalización: El OCR entrega los números.
+2.	Transformación: Los números se convierten en curvas de energía ($K/S$).
+3.	Comparación Vectorial: Se mide la distancia entre el estándar y el lote dentro del elipsoide de tolerancia.
+4.	Traducción Química: Esa distancia se traduce a porcentaje de colorante ($\Delta\%$) y finalmente a la recomendación de ingeniería que ves en la pantalla final.</t>
   </si>
 </sst>
 </file>
@@ -409,7 +584,7 @@
     <numFmt numFmtId="167" formatCode="0.00000"/>
     <numFmt numFmtId="168" formatCode="0.000000"/>
   </numFmts>
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -505,6 +680,56 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="7"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Segoe UI Symbol"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -538,7 +763,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -627,11 +852,36 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="14" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="81">
+  <cellXfs count="97">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -762,6 +1012,44 @@
     <xf numFmtId="9" fontId="9" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="5"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -774,12 +1062,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="2" fontId="8" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -813,27 +1095,27 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -843,9 +1125,22 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -858,6 +1153,579 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>609600</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>19050</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="2" name="Straight Arrow Connector 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9A036C56-3AA8-4812-A378-E9E2966DC91F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="609600" y="7620000"/>
+          <a:ext cx="876300" cy="190500"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>571500</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>28575</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="3" name="Straight Arrow Connector 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4A3EC302-F39C-47B8-A208-2515A9C52782}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="571500" y="7810500"/>
+          <a:ext cx="923925" cy="219075"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>152400</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>285750</xdr:colOff>
+      <xdr:row>43</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="4" name="Straight Arrow Connector 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{131057BE-94F2-461A-881A-47D5287DDF76}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2190750" y="8039100"/>
+          <a:ext cx="704850" cy="266700"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>209550</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>43</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="5" name="Straight Arrow Connector 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BC2A0F86-4407-4382-9834-77D8CEE39FEA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1">
+          <a:off x="1676400" y="8020050"/>
+          <a:ext cx="361950" cy="333375"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>371475</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>342900</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>180975</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="6" name="Arrow: Right 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4F0159DB-27BF-4085-9F1C-214BB34B493C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2981325" y="7429500"/>
+          <a:ext cx="1457325" cy="228600"/>
+        </a:xfrm>
+        <a:prstGeom prst="rightArrow">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="es-CO" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>712615</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>121756</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>207648</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>30833</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="7" name="Arrow: Right 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A97DA82C-D1AC-4E8C-835E-A5555789F8D2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="8132590" y="7598881"/>
+          <a:ext cx="1066658" cy="328177"/>
+        </a:xfrm>
+        <a:prstGeom prst="rightArrow">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="es-CO" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1273175</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>62442</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>68792</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>3175</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="8" name="Right Bracket 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EC385C18-FF22-4255-AD8B-2DB2ACC26C72}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7302500" y="7120467"/>
+          <a:ext cx="186267" cy="359833"/>
+        </a:xfrm>
+        <a:prstGeom prst="rightBracket">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="es-CO" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1261533</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>49741</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>202141</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="9" name="Right Bracket 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D9076EC7-6620-40E0-8522-5F2194AF656F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7290858" y="7526866"/>
+          <a:ext cx="167217" cy="361950"/>
+        </a:xfrm>
+        <a:prstGeom prst="rightBracket">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="es-CO" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>596198</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>68841</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>122982</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>189584</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="10" name="Arrow: Right 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3179BF79-080F-423F-AFDE-D8EC7299F772}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="8016173" y="7126866"/>
+          <a:ext cx="1098409" cy="330293"/>
+        </a:xfrm>
+        <a:prstGeom prst="rightArrow">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="es-CO" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>656166</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>21167</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>690950</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>141910</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="11" name="Arrow: Right 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{455ABC7C-5BBB-4EE4-8FDC-A3FA8D2FB076}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="11095566" y="7288742"/>
+          <a:ext cx="1073009" cy="330293"/>
+        </a:xfrm>
+        <a:prstGeom prst="rightArrow">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="es-CO" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1268,16 +2136,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7BE2DF79-A7C0-4C59-8A5D-80E5B6D3C3CA}">
-  <dimension ref="A1:U29"/>
+  <dimension ref="A1:U44"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="16.42578125" customWidth="1"/>
-    <col min="3" max="3" width="17.7109375" customWidth="1"/>
-    <col min="4" max="4" width="19.7109375" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="15.85546875" customWidth="1"/>
+    <col min="4" max="5" width="11.140625" customWidth="1"/>
     <col min="6" max="6" width="20.42578125" customWidth="1"/>
-    <col min="9" max="9" width="33" customWidth="1"/>
+    <col min="8" max="8" width="20.85546875" customWidth="1"/>
+    <col min="9" max="9" width="12" customWidth="1"/>
     <col min="10" max="10" width="11.5703125" customWidth="1"/>
     <col min="11" max="11" width="10.5703125" customWidth="1"/>
     <col min="12" max="12" width="11.140625" customWidth="1"/>
@@ -1291,13 +2157,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="54" t="s">
-        <v>103</v>
-      </c>
-      <c r="B1" s="54"/>
-      <c r="C1" s="54"/>
-      <c r="D1" s="54"/>
-      <c r="E1" s="54"/>
+      <c r="A1" s="68" t="s">
+        <v>107</v>
+      </c>
+      <c r="B1" s="68"/>
+      <c r="C1" s="68"/>
+      <c r="D1" s="68"/>
+      <c r="E1" s="68"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
@@ -1312,14 +2178,16 @@
       </c>
       <c r="D2" s="2"/>
       <c r="E2" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="F2" s="1"/>
+        <v>108</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>136</v>
+      </c>
       <c r="G2" s="1"/>
-      <c r="H2" s="57" t="s">
+      <c r="H2" s="71" t="s">
         <v>27</v>
       </c>
-      <c r="I2" s="57"/>
+      <c r="I2" s="71"/>
       <c r="J2" s="11"/>
       <c r="K2" s="11"/>
       <c r="L2" s="11"/>
@@ -1328,33 +2196,36 @@
     </row>
     <row r="3" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>31</v>
+        <v>109</v>
       </c>
       <c r="B3" s="33">
         <v>82.83</v>
       </c>
       <c r="C3" s="33">
-        <v>80.680000000000007</v>
-      </c>
-      <c r="D3" s="12">
+        <v>80.599999999999994</v>
+      </c>
+      <c r="D3" s="54">
         <f>+(B3-C3)/B3</f>
-        <v>2.5956778944826651E-2</v>
-      </c>
-      <c r="E3" s="12">
+        <v>2.6922612579983147E-2</v>
+      </c>
+      <c r="E3" s="54">
         <f>+ABS(D3)</f>
-        <v>2.5956778944826651E-2</v>
-      </c>
-      <c r="F3" s="1"/>
+        <v>2.6922612579983147E-2</v>
+      </c>
+      <c r="F3" s="55">
+        <f>E3/100%</f>
+        <v>2.6922612579983147E-2</v>
+      </c>
       <c r="G3" s="1"/>
       <c r="H3" s="13">
         <f>+E3/B3</f>
-        <v>3.1337412706539483E-4</v>
+        <v>3.2503455970038812E-4</v>
       </c>
       <c r="I3" s="2" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:21" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>101</v>
       </c>
@@ -1372,7 +2243,10 @@
         <f>+ABS(D4)</f>
         <v>8.6376404494382053E-2</v>
       </c>
-      <c r="F4" s="1"/>
+      <c r="F4" s="55">
+        <f>E4/100%</f>
+        <v>8.6376404494382053E-2</v>
+      </c>
       <c r="G4" s="1"/>
       <c r="H4" s="13">
         <f>+E4/B4</f>
@@ -1382,7 +2256,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>102</v>
       </c>
@@ -1392,7 +2266,7 @@
       <c r="C5" s="33">
         <v>-3.47</v>
       </c>
-      <c r="D5" s="12">
+      <c r="D5" s="56">
         <f>+(B5-C5)/B5</f>
         <v>3.611111111111108E-2</v>
       </c>
@@ -1400,7 +2274,10 @@
         <f>+ABS(D5)</f>
         <v>3.611111111111108E-2</v>
       </c>
-      <c r="F5" s="1"/>
+      <c r="F5" s="55">
+        <f>E5/100%</f>
+        <v>3.611111111111108E-2</v>
+      </c>
       <c r="G5" s="1"/>
       <c r="H5" s="13">
         <f>+E5/B5</f>
@@ -1410,7 +2287,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:21" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="6" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="7" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
         <v>53</v>
@@ -1437,6 +2314,10 @@
         <f>MOD(ATAN2(B4,B5)*180/PI(),360)</f>
         <v>194.18761901931759</v>
       </c>
+      <c r="F9" s="57">
+        <f>E4/(1-E4)</f>
+        <v>9.4542659492697953E-2</v>
+      </c>
     </row>
     <row r="10" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
@@ -1465,11 +2346,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="14"/>
       <c r="B13" s="15"/>
     </row>
-    <row r="14" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="7"/>
       <c r="C14" s="7"/>
       <c r="D14" s="7" t="s">
@@ -1527,8 +2408,8 @@
         <v>58</v>
       </c>
     </row>
-    <row r="15" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="55" t="s">
+    <row r="15" spans="1:21" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="69" t="s">
         <v>6</v>
       </c>
       <c r="C15" s="7" t="s">
@@ -1543,39 +2424,39 @@
       <c r="F15" s="28">
         <v>-3.6</v>
       </c>
-      <c r="G15" s="58">
+      <c r="G15" s="69">
         <f>+(D15-D16)/D15</f>
         <v>2.5956778944826651E-2</v>
       </c>
-      <c r="H15" s="59">
+      <c r="H15" s="69">
         <f>+(E15-E16)/E15</f>
         <v>8.6376404494382053E-2</v>
       </c>
-      <c r="I15" s="58">
+      <c r="I15" s="69">
         <f>+(F15-F16)/F15</f>
         <v>3.611111111111108E-2</v>
       </c>
-      <c r="J15" s="58">
+      <c r="J15" s="69">
         <f>+ABS(G15)</f>
         <v>2.5956778944826651E-2</v>
       </c>
-      <c r="K15" s="58">
+      <c r="K15" s="69">
         <f>+ABS(H15)</f>
         <v>8.6376404494382053E-2</v>
       </c>
-      <c r="L15" s="55">
+      <c r="L15" s="69">
         <f>+ABS(I15)</f>
         <v>3.611111111111108E-2</v>
       </c>
-      <c r="M15" s="56">
+      <c r="M15" s="70">
         <f>+K15/F15</f>
         <v>-2.3993445692883902E-2</v>
       </c>
-      <c r="N15" s="56">
+      <c r="N15" s="70">
         <f>+K15/E15</f>
         <v>-6.0657587425830091E-3</v>
       </c>
-      <c r="O15" s="56">
+      <c r="O15" s="70">
         <f>+L15/F15</f>
         <v>-1.0030864197530855E-2</v>
       </c>
@@ -1604,8 +2485,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="55"/>
+    <row r="16" spans="1:21" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="69"/>
       <c r="C16" s="7" t="s">
         <v>26</v>
       </c>
@@ -1618,15 +2499,15 @@
       <c r="F16" s="28">
         <v>-3.47</v>
       </c>
-      <c r="G16" s="58"/>
-      <c r="H16" s="59"/>
-      <c r="I16" s="58"/>
-      <c r="J16" s="58"/>
-      <c r="K16" s="58"/>
-      <c r="L16" s="55"/>
-      <c r="M16" s="55"/>
-      <c r="N16" s="55"/>
-      <c r="O16" s="55"/>
+      <c r="G16" s="69"/>
+      <c r="H16" s="69"/>
+      <c r="I16" s="69"/>
+      <c r="J16" s="69"/>
+      <c r="K16" s="69"/>
+      <c r="L16" s="69"/>
+      <c r="M16" s="69"/>
+      <c r="N16" s="69"/>
+      <c r="O16" s="69"/>
       <c r="P16" s="7"/>
       <c r="Q16" s="7"/>
       <c r="R16" s="7"/>
@@ -1634,8 +2515,8 @@
       <c r="T16" s="7"/>
       <c r="U16" s="7"/>
     </row>
-    <row r="17" spans="2:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="55" t="s">
+    <row r="17" spans="2:21" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="69" t="s">
         <v>7</v>
       </c>
       <c r="C17" s="7" t="s">
@@ -1650,39 +2531,39 @@
       <c r="F17" s="28">
         <v>5.0599999999999996</v>
       </c>
-      <c r="G17" s="58">
+      <c r="G17" s="69">
         <f>+(D17-D18)/D17</f>
         <v>2.4813592470358161E-2</v>
       </c>
-      <c r="H17" s="59">
+      <c r="H17" s="69">
         <f>+(E17-E18)/E17</f>
         <v>5.7165231010180145E-2</v>
       </c>
-      <c r="I17" s="59">
+      <c r="I17" s="69">
         <f>+(F17-F18)/F17</f>
         <v>1.8557312252964429</v>
       </c>
-      <c r="J17" s="58">
+      <c r="J17" s="69">
         <f>+ABS(G17)</f>
         <v>2.4813592470358161E-2</v>
       </c>
-      <c r="K17" s="55">
+      <c r="K17" s="69">
         <f>+ABS(H17)</f>
         <v>5.7165231010180145E-2</v>
       </c>
-      <c r="L17" s="55">
+      <c r="L17" s="69">
         <f>+ABS(I17)</f>
         <v>1.8557312252964429</v>
       </c>
-      <c r="M17" s="56">
+      <c r="M17" s="70">
         <f>+J17/D17</f>
         <v>3.0330757206158365E-4</v>
       </c>
-      <c r="N17" s="56">
+      <c r="N17" s="70">
         <f>+K17/E17</f>
         <v>-4.4765255293798076E-3</v>
       </c>
-      <c r="O17" s="56">
+      <c r="O17" s="70">
         <f>+L17/F17</f>
         <v>0.36674530144198481</v>
       </c>
@@ -1711,8 +2592,8 @@
         <v>1.6004671261736865</v>
       </c>
     </row>
-    <row r="18" spans="2:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="55"/>
+    <row r="18" spans="2:21" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="69"/>
       <c r="C18" s="7" t="s">
         <v>26</v>
       </c>
@@ -1725,15 +2606,15 @@
       <c r="F18" s="28">
         <v>-4.33</v>
       </c>
-      <c r="G18" s="58"/>
-      <c r="H18" s="59"/>
-      <c r="I18" s="59"/>
-      <c r="J18" s="58"/>
-      <c r="K18" s="55"/>
-      <c r="L18" s="55"/>
-      <c r="M18" s="55"/>
-      <c r="N18" s="55"/>
-      <c r="O18" s="55"/>
+      <c r="G18" s="69"/>
+      <c r="H18" s="69"/>
+      <c r="I18" s="69"/>
+      <c r="J18" s="69"/>
+      <c r="K18" s="69"/>
+      <c r="L18" s="69"/>
+      <c r="M18" s="69"/>
+      <c r="N18" s="69"/>
+      <c r="O18" s="69"/>
       <c r="P18" s="7"/>
       <c r="Q18" s="7"/>
       <c r="R18" s="7"/>
@@ -1741,8 +2622,8 @@
       <c r="T18" s="7"/>
       <c r="U18" s="7"/>
     </row>
-    <row r="19" spans="2:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="55" t="s">
+    <row r="19" spans="2:21" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="69" t="s">
         <v>32</v>
       </c>
       <c r="C19" s="7" t="s">
@@ -1757,39 +2638,39 @@
       <c r="F19" s="28">
         <v>7.39</v>
       </c>
-      <c r="G19" s="58">
+      <c r="G19" s="69">
         <f>+(D19-D20)/D19</f>
         <v>4.9419322955275513E-2</v>
       </c>
-      <c r="H19" s="59">
+      <c r="H19" s="69">
         <f>+(E19-E20)/E19</f>
         <v>5.7884231536926095E-2</v>
       </c>
-      <c r="I19" s="58">
+      <c r="I19" s="69">
         <f>+(F19-F20)/F19</f>
         <v>7.9837618403247615E-2</v>
       </c>
-      <c r="J19" s="58">
+      <c r="J19" s="69">
         <f>+ABS(G19)</f>
         <v>4.9419322955275513E-2</v>
       </c>
-      <c r="K19" s="55">
+      <c r="K19" s="69">
         <f>+ABS(H19)</f>
         <v>5.7884231536926095E-2</v>
       </c>
-      <c r="L19" s="55">
+      <c r="L19" s="69">
         <f>+ABS(I19)</f>
         <v>7.9837618403247615E-2</v>
       </c>
-      <c r="M19" s="56">
+      <c r="M19" s="70">
         <f>+J19/D19</f>
         <v>6.1056737033945529E-4</v>
       </c>
-      <c r="N19" s="56">
+      <c r="N19" s="70">
         <f>+K19/E19</f>
         <v>-3.8512462765752562E-3</v>
       </c>
-      <c r="O19" s="56">
+      <c r="O19" s="70">
         <f>+L19/F19</f>
         <v>1.0803466631021328E-2</v>
       </c>
@@ -1818,8 +2699,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="2:21" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="55"/>
+    <row r="20" spans="2:21" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="69"/>
       <c r="C20" s="7" t="s">
         <v>26</v>
       </c>
@@ -1832,15 +2713,15 @@
       <c r="F20" s="28">
         <v>6.8</v>
       </c>
-      <c r="G20" s="58"/>
-      <c r="H20" s="59"/>
-      <c r="I20" s="58"/>
-      <c r="J20" s="58"/>
-      <c r="K20" s="55"/>
-      <c r="L20" s="55"/>
-      <c r="M20" s="55"/>
-      <c r="N20" s="55"/>
-      <c r="O20" s="55"/>
+      <c r="G20" s="69"/>
+      <c r="H20" s="69"/>
+      <c r="I20" s="69"/>
+      <c r="J20" s="69"/>
+      <c r="K20" s="69"/>
+      <c r="L20" s="69"/>
+      <c r="M20" s="69"/>
+      <c r="N20" s="69"/>
+      <c r="O20" s="69"/>
       <c r="P20" s="7"/>
       <c r="Q20" s="7"/>
       <c r="R20" s="7"/>
@@ -1848,8 +2729,8 @@
       <c r="T20" s="7"/>
       <c r="U20" s="7"/>
     </row>
-    <row r="21" spans="2:21" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="22" spans="2:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:21" ht="30.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="22" spans="2:21" ht="57" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="7" t="s">
         <v>31</v>
       </c>
@@ -1860,59 +2741,184 @@
         <v>33</v>
       </c>
     </row>
-    <row r="23" spans="2:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:21" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="24" spans="2:21" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="7"/>
+      <c r="C24" s="7"/>
+      <c r="D24" s="7"/>
+    </row>
+    <row r="25" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B25" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="37" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="38" spans="1:18" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F38" s="58" t="s">
+        <v>112</v>
+      </c>
+      <c r="I38" s="67" t="s">
+        <v>113</v>
+      </c>
+      <c r="L38" t="s">
+        <v>114</v>
+      </c>
+      <c r="M38" s="59"/>
+      <c r="N38" s="59"/>
+      <c r="O38" s="60" t="s">
+        <v>79</v>
+      </c>
+      <c r="P38" s="61" t="s">
+        <v>115</v>
+      </c>
+      <c r="Q38" s="61" t="s">
+        <v>116</v>
+      </c>
+      <c r="R38" s="61" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="39" spans="1:18" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B39" t="s">
+        <v>104</v>
+      </c>
+      <c r="C39" t="s">
+        <v>105</v>
+      </c>
+      <c r="D39" t="s">
         <v>106</v>
       </c>
-      <c r="C23" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="D23" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="I23" t="s">
-        <v>105</v>
-      </c>
-      <c r="J23" t="s">
-        <v>101</v>
-      </c>
-      <c r="K23" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="24" spans="2:21" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="29" spans="2:21" x14ac:dyDescent="0.25">
-      <c r="N29" t="s">
-        <v>107</v>
-      </c>
-      <c r="O29" t="s">
-        <v>108</v>
-      </c>
-      <c r="P29" t="s">
-        <v>109</v>
+      <c r="F39" s="58" t="s">
+        <v>118</v>
+      </c>
+      <c r="I39" s="67"/>
+      <c r="L39" t="s">
+        <v>119</v>
+      </c>
+      <c r="M39" s="62"/>
+      <c r="N39" s="62"/>
+      <c r="O39" s="63" t="s">
+        <v>32</v>
+      </c>
+      <c r="P39" s="64" t="s">
+        <v>120</v>
+      </c>
+      <c r="Q39" s="64" t="s">
+        <v>121</v>
+      </c>
+      <c r="R39" s="63" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="40" spans="1:18" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>123</v>
+      </c>
+      <c r="B40" t="s">
+        <v>124</v>
+      </c>
+      <c r="C40" t="s">
+        <v>124</v>
+      </c>
+      <c r="D40" t="s">
+        <v>124</v>
+      </c>
+      <c r="F40" s="58" t="s">
+        <v>125</v>
+      </c>
+      <c r="I40" s="67" t="s">
+        <v>126</v>
+      </c>
+      <c r="L40" t="s">
+        <v>127</v>
+      </c>
+      <c r="M40" s="62"/>
+      <c r="N40" s="62"/>
+      <c r="O40" s="63" t="s">
+        <v>33</v>
+      </c>
+      <c r="P40" s="64" t="s">
+        <v>128</v>
+      </c>
+      <c r="Q40" s="64" t="s">
+        <v>120</v>
+      </c>
+      <c r="R40" s="65"/>
+    </row>
+    <row r="41" spans="1:18" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B41" t="s">
+        <v>129</v>
+      </c>
+      <c r="C41" t="s">
+        <v>124</v>
+      </c>
+      <c r="D41" t="s">
+        <v>124</v>
+      </c>
+      <c r="F41" s="58" t="s">
+        <v>130</v>
+      </c>
+      <c r="I41" s="67"/>
+      <c r="L41" t="s">
+        <v>131</v>
+      </c>
+      <c r="M41" s="62"/>
+      <c r="N41" s="62"/>
+      <c r="O41" s="66" t="s">
+        <v>132</v>
+      </c>
+      <c r="P41" s="64" t="s">
+        <v>121</v>
+      </c>
+      <c r="Q41" s="64" t="s">
+        <v>121</v>
+      </c>
+      <c r="R41" s="64" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="42" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>133</v>
+      </c>
+      <c r="B42" t="s">
+        <v>124</v>
+      </c>
+      <c r="C42" t="s">
+        <v>129</v>
+      </c>
+      <c r="D42" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="44" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="B44" t="s">
+        <v>134</v>
+      </c>
+      <c r="D44" t="s">
+        <v>135</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="32">
-    <mergeCell ref="K15:K16"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="G19:G20"/>
-    <mergeCell ref="H19:H20"/>
-    <mergeCell ref="I19:I20"/>
-    <mergeCell ref="J19:J20"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="G17:G18"/>
-    <mergeCell ref="H17:H18"/>
-    <mergeCell ref="I17:I18"/>
-    <mergeCell ref="J17:J18"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="G15:G16"/>
-    <mergeCell ref="H15:H16"/>
+  <mergeCells count="34">
     <mergeCell ref="I15:I16"/>
     <mergeCell ref="J15:J16"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="L19:L20"/>
-    <mergeCell ref="M19:M20"/>
     <mergeCell ref="N19:N20"/>
     <mergeCell ref="O19:O20"/>
     <mergeCell ref="H2:I2"/>
@@ -1926,8 +2932,28 @@
     <mergeCell ref="N15:N16"/>
     <mergeCell ref="O15:O16"/>
     <mergeCell ref="K17:K18"/>
+    <mergeCell ref="K15:K16"/>
+    <mergeCell ref="H19:H20"/>
+    <mergeCell ref="I19:I20"/>
+    <mergeCell ref="I38:I39"/>
+    <mergeCell ref="I40:I41"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="L19:L20"/>
+    <mergeCell ref="M19:M20"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="G19:G20"/>
+    <mergeCell ref="J19:J20"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="G17:G18"/>
+    <mergeCell ref="H17:H18"/>
+    <mergeCell ref="I17:I18"/>
+    <mergeCell ref="J17:J18"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="G15:G16"/>
+    <mergeCell ref="H15:H16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1954,13 +2980,13 @@
   </cols>
   <sheetData>
     <row r="2" spans="4:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E2" s="57" t="s">
+      <c r="E2" s="71" t="s">
         <v>48</v>
       </c>
-      <c r="F2" s="57"/>
-      <c r="G2" s="57"/>
-      <c r="H2" s="57"/>
-      <c r="I2" s="57"/>
+      <c r="F2" s="71"/>
+      <c r="G2" s="71"/>
+      <c r="H2" s="71"/>
+      <c r="I2" s="71"/>
     </row>
     <row r="3" spans="4:15" x14ac:dyDescent="0.2">
       <c r="E3" s="2"/>
@@ -2008,30 +3034,30 @@
       <c r="O4" s="2"/>
     </row>
     <row r="5" spans="4:15" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E5" s="68" t="s">
+      <c r="E5" s="80" t="s">
         <v>6</v>
       </c>
-      <c r="F5" s="65">
+      <c r="F5" s="77">
         <v>-0.78</v>
       </c>
-      <c r="G5" s="65">
+      <c r="G5" s="77">
         <v>-0.86</v>
       </c>
-      <c r="H5" s="67">
+      <c r="H5" s="79">
         <v>0.17</v>
       </c>
-      <c r="I5" s="63">
+      <c r="I5" s="75">
         <v>1.17</v>
       </c>
-      <c r="J5" s="72">
+      <c r="J5" s="87">
         <f>+ABS(F5*10)</f>
         <v>7.8000000000000007</v>
       </c>
-      <c r="K5" s="74">
+      <c r="K5" s="86">
         <f>+ABS(G5*10)</f>
         <v>8.6</v>
       </c>
-      <c r="L5" s="74">
+      <c r="L5" s="86">
         <f>+ABS(H5*10)</f>
         <v>1.7000000000000002</v>
       </c>
@@ -2049,43 +3075,43 @@
       </c>
     </row>
     <row r="6" spans="4:15" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E6" s="68"/>
-      <c r="F6" s="66"/>
-      <c r="G6" s="66"/>
-      <c r="H6" s="66"/>
-      <c r="I6" s="64"/>
-      <c r="J6" s="72"/>
-      <c r="K6" s="74"/>
-      <c r="L6" s="74"/>
+      <c r="E6" s="80"/>
+      <c r="F6" s="78"/>
+      <c r="G6" s="78"/>
+      <c r="H6" s="78"/>
+      <c r="I6" s="76"/>
+      <c r="J6" s="87"/>
+      <c r="K6" s="86"/>
+      <c r="L6" s="86"/>
       <c r="M6" s="2"/>
       <c r="N6" s="2"/>
       <c r="O6" s="2"/>
     </row>
     <row r="7" spans="4:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E7" s="57" t="s">
+      <c r="E7" s="71" t="s">
         <v>7</v>
       </c>
-      <c r="F7" s="60">
+      <c r="F7" s="72">
         <v>-0.74</v>
       </c>
-      <c r="G7" s="62">
+      <c r="G7" s="74">
         <v>-0.54</v>
       </c>
-      <c r="H7" s="62">
+      <c r="H7" s="74">
         <v>0.1</v>
       </c>
-      <c r="I7" s="61">
+      <c r="I7" s="73">
         <v>0.92</v>
       </c>
-      <c r="J7" s="73">
+      <c r="J7" s="88">
         <f>+ABS(F7*10)</f>
         <v>7.4</v>
       </c>
-      <c r="K7" s="71">
+      <c r="K7" s="89">
         <f>+ABS(G7*10)</f>
         <v>5.4</v>
       </c>
-      <c r="L7" s="71">
+      <c r="L7" s="89">
         <f>+ABS(H7*10)</f>
         <v>1</v>
       </c>
@@ -2103,43 +3129,43 @@
       </c>
     </row>
     <row r="8" spans="4:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E8" s="57"/>
-      <c r="F8" s="61"/>
-      <c r="G8" s="61"/>
-      <c r="H8" s="61"/>
-      <c r="I8" s="61"/>
-      <c r="J8" s="73"/>
-      <c r="K8" s="71"/>
-      <c r="L8" s="71"/>
+      <c r="E8" s="71"/>
+      <c r="F8" s="73"/>
+      <c r="G8" s="73"/>
+      <c r="H8" s="73"/>
+      <c r="I8" s="73"/>
+      <c r="J8" s="88"/>
+      <c r="K8" s="89"/>
+      <c r="L8" s="89"/>
       <c r="M8" s="2"/>
       <c r="N8" s="2"/>
       <c r="O8" s="2"/>
     </row>
     <row r="9" spans="4:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E9" s="57" t="s">
+      <c r="E9" s="71" t="s">
         <v>8</v>
       </c>
-      <c r="F9" s="60">
+      <c r="F9" s="72">
         <v>-0.73</v>
       </c>
-      <c r="G9" s="62">
+      <c r="G9" s="74">
         <v>-0.68</v>
       </c>
-      <c r="H9" s="62">
+      <c r="H9" s="74">
         <v>-0.12</v>
       </c>
-      <c r="I9" s="61">
+      <c r="I9" s="73">
         <v>1.01</v>
       </c>
-      <c r="J9" s="73">
+      <c r="J9" s="88">
         <f>+ABS(F9*10)</f>
         <v>7.3</v>
       </c>
-      <c r="K9" s="71">
+      <c r="K9" s="89">
         <f>+ABS(G9*10)</f>
         <v>6.8000000000000007</v>
       </c>
-      <c r="L9" s="71">
+      <c r="L9" s="89">
         <f>+ABS(H9*10)</f>
         <v>1.2</v>
       </c>
@@ -2157,14 +3183,14 @@
       </c>
     </row>
     <row r="10" spans="4:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E10" s="57"/>
-      <c r="F10" s="61"/>
-      <c r="G10" s="61"/>
-      <c r="H10" s="61"/>
-      <c r="I10" s="61"/>
-      <c r="J10" s="73"/>
-      <c r="K10" s="71"/>
-      <c r="L10" s="71"/>
+      <c r="E10" s="71"/>
+      <c r="F10" s="73"/>
+      <c r="G10" s="73"/>
+      <c r="H10" s="73"/>
+      <c r="I10" s="73"/>
+      <c r="J10" s="88"/>
+      <c r="K10" s="89"/>
+      <c r="L10" s="89"/>
       <c r="M10" s="2"/>
       <c r="N10" s="2"/>
       <c r="O10" s="2"/>
@@ -2175,51 +3201,51 @@
       <c r="H11" s="9"/>
     </row>
     <row r="12" spans="4:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E12" s="75" t="s">
+      <c r="E12" s="83" t="s">
         <v>46</v>
       </c>
-      <c r="F12" s="76"/>
-      <c r="G12" s="76"/>
-      <c r="H12" s="76"/>
-      <c r="I12" s="76"/>
-      <c r="J12" s="76"/>
-      <c r="K12" s="76"/>
-      <c r="L12" s="76"/>
-      <c r="M12" s="76"/>
-      <c r="N12" s="76"/>
-      <c r="O12" s="77"/>
+      <c r="F12" s="84"/>
+      <c r="G12" s="84"/>
+      <c r="H12" s="84"/>
+      <c r="I12" s="84"/>
+      <c r="J12" s="84"/>
+      <c r="K12" s="84"/>
+      <c r="L12" s="84"/>
+      <c r="M12" s="84"/>
+      <c r="N12" s="84"/>
+      <c r="O12" s="85"/>
     </row>
     <row r="13" spans="4:15" x14ac:dyDescent="0.25">
-      <c r="E13" s="57" t="s">
+      <c r="E13" s="71" t="s">
         <v>47</v>
       </c>
-      <c r="F13" s="57"/>
-      <c r="G13" s="57"/>
-      <c r="H13" s="57"/>
-      <c r="I13" s="57"/>
-      <c r="J13" s="75" t="s">
+      <c r="F13" s="71"/>
+      <c r="G13" s="71"/>
+      <c r="H13" s="71"/>
+      <c r="I13" s="71"/>
+      <c r="J13" s="83" t="s">
         <v>19</v>
       </c>
-      <c r="K13" s="76"/>
-      <c r="L13" s="76"/>
-      <c r="M13" s="76"/>
-      <c r="N13" s="76"/>
-      <c r="O13" s="77"/>
+      <c r="K13" s="84"/>
+      <c r="L13" s="84"/>
+      <c r="M13" s="84"/>
+      <c r="N13" s="84"/>
+      <c r="O13" s="85"/>
     </row>
     <row r="14" spans="4:15" x14ac:dyDescent="0.2">
       <c r="E14" s="2"/>
-      <c r="F14" s="57" t="s">
+      <c r="F14" s="71" t="s">
         <v>49</v>
       </c>
-      <c r="G14" s="57"/>
-      <c r="H14" s="57" t="s">
+      <c r="G14" s="71"/>
+      <c r="H14" s="71" t="s">
         <v>43</v>
       </c>
-      <c r="I14" s="57"/>
-      <c r="J14" s="57" t="s">
+      <c r="I14" s="71"/>
+      <c r="J14" s="71" t="s">
         <v>17</v>
       </c>
-      <c r="K14" s="57"/>
+      <c r="K14" s="71"/>
       <c r="L14" s="2"/>
       <c r="M14" s="26" t="s">
         <v>63</v>
@@ -2232,7 +3258,7 @@
       </c>
     </row>
     <row r="15" spans="4:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D15" s="69"/>
+      <c r="D15" s="81"/>
       <c r="E15" s="29" t="s">
         <v>12</v>
       </c>
@@ -2269,7 +3295,7 @@
       <c r="O15" s="26"/>
     </row>
     <row r="16" spans="4:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D16" s="69"/>
+      <c r="D16" s="81"/>
       <c r="E16" s="29" t="s">
         <v>13</v>
       </c>
@@ -2302,7 +3328,7 @@
       <c r="O16" s="2"/>
     </row>
     <row r="17" spans="4:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D17" s="69"/>
+      <c r="D17" s="81"/>
       <c r="E17" s="29" t="s">
         <v>14</v>
       </c>
@@ -2335,7 +3361,7 @@
       <c r="O17" s="2"/>
     </row>
     <row r="18" spans="4:17" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D18" s="69"/>
+      <c r="D18" s="81"/>
       <c r="E18" s="2" t="s">
         <v>15</v>
       </c>
@@ -2378,7 +3404,7 @@
       </c>
     </row>
     <row r="19" spans="4:17" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D19" s="69"/>
+      <c r="D19" s="81"/>
       <c r="E19" s="2" t="s">
         <v>16</v>
       </c>
@@ -2401,41 +3427,41 @@
       <c r="P19" s="27"/>
     </row>
     <row r="21" spans="4:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E21" s="70" t="s">
+      <c r="E21" s="82" t="s">
         <v>50</v>
       </c>
-      <c r="F21" s="54"/>
-      <c r="G21" s="54"/>
-      <c r="H21" s="54"/>
-      <c r="I21" s="54"/>
-      <c r="J21" s="54"/>
-      <c r="K21" s="54"/>
-      <c r="L21" s="54"/>
-      <c r="M21" s="54"/>
-      <c r="N21" s="54"/>
-      <c r="O21" s="54"/>
-      <c r="P21" s="54"/>
-      <c r="Q21" s="54"/>
+      <c r="F21" s="68"/>
+      <c r="G21" s="68"/>
+      <c r="H21" s="68"/>
+      <c r="I21" s="68"/>
+      <c r="J21" s="68"/>
+      <c r="K21" s="68"/>
+      <c r="L21" s="68"/>
+      <c r="M21" s="68"/>
+      <c r="N21" s="68"/>
+      <c r="O21" s="68"/>
+      <c r="P21" s="68"/>
+      <c r="Q21" s="68"/>
     </row>
     <row r="22" spans="4:17" x14ac:dyDescent="0.2">
       <c r="E22" s="2"/>
-      <c r="F22" s="57" t="s">
+      <c r="F22" s="71" t="s">
         <v>9</v>
       </c>
-      <c r="G22" s="57"/>
-      <c r="H22" s="57" t="s">
+      <c r="G22" s="71"/>
+      <c r="H22" s="71" t="s">
         <v>10</v>
       </c>
-      <c r="I22" s="57"/>
-      <c r="J22" s="57" t="s">
+      <c r="I22" s="71"/>
+      <c r="J22" s="71" t="s">
         <v>11</v>
       </c>
-      <c r="K22" s="57"/>
+      <c r="K22" s="71"/>
       <c r="L22" s="2"/>
-      <c r="M22" s="57" t="s">
+      <c r="M22" s="71" t="s">
         <v>70</v>
       </c>
-      <c r="N22" s="57"/>
+      <c r="N22" s="71"/>
       <c r="O22" s="26" t="s">
         <v>55</v>
       </c>
@@ -2447,7 +3473,7 @@
       </c>
     </row>
     <row r="23" spans="4:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D23" s="69"/>
+      <c r="D23" s="81"/>
       <c r="E23" s="29" t="s">
         <v>12</v>
       </c>
@@ -2488,7 +3514,7 @@
       <c r="Q23" s="2"/>
     </row>
     <row r="24" spans="4:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D24" s="69"/>
+      <c r="D24" s="81"/>
       <c r="E24" s="29" t="s">
         <v>13</v>
       </c>
@@ -2529,7 +3555,7 @@
       <c r="Q24" s="2"/>
     </row>
     <row r="25" spans="4:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D25" s="69"/>
+      <c r="D25" s="81"/>
       <c r="E25" s="29" t="s">
         <v>14</v>
       </c>
@@ -2570,7 +3596,7 @@
       <c r="Q25" s="2"/>
     </row>
     <row r="26" spans="4:17" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D26" s="69"/>
+      <c r="D26" s="81"/>
       <c r="E26" s="2" t="s">
         <v>15</v>
       </c>
@@ -2621,7 +3647,7 @@
       </c>
     </row>
     <row r="27" spans="4:17" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D27" s="69"/>
+      <c r="D27" s="81"/>
       <c r="E27" s="2" t="s">
         <v>16</v>
       </c>
@@ -2655,41 +3681,41 @@
       <c r="Q27" s="2"/>
     </row>
     <row r="29" spans="4:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E29" s="70" t="s">
+      <c r="E29" s="82" t="s">
         <v>51</v>
       </c>
-      <c r="F29" s="54"/>
-      <c r="G29" s="54"/>
-      <c r="H29" s="54"/>
-      <c r="I29" s="54"/>
-      <c r="J29" s="54"/>
-      <c r="K29" s="54"/>
-      <c r="L29" s="54"/>
-      <c r="M29" s="54"/>
-      <c r="N29" s="54"/>
-      <c r="O29" s="54"/>
-      <c r="P29" s="54"/>
-      <c r="Q29" s="54"/>
+      <c r="F29" s="68"/>
+      <c r="G29" s="68"/>
+      <c r="H29" s="68"/>
+      <c r="I29" s="68"/>
+      <c r="J29" s="68"/>
+      <c r="K29" s="68"/>
+      <c r="L29" s="68"/>
+      <c r="M29" s="68"/>
+      <c r="N29" s="68"/>
+      <c r="O29" s="68"/>
+      <c r="P29" s="68"/>
+      <c r="Q29" s="68"/>
     </row>
     <row r="30" spans="4:17" ht="25.5" x14ac:dyDescent="0.2">
       <c r="E30" s="2"/>
-      <c r="F30" s="57" t="s">
+      <c r="F30" s="71" t="s">
         <v>9</v>
       </c>
-      <c r="G30" s="57"/>
-      <c r="H30" s="57" t="s">
+      <c r="G30" s="71"/>
+      <c r="H30" s="71" t="s">
         <v>10</v>
       </c>
-      <c r="I30" s="57"/>
-      <c r="J30" s="57" t="s">
+      <c r="I30" s="71"/>
+      <c r="J30" s="71" t="s">
         <v>11</v>
       </c>
-      <c r="K30" s="57"/>
+      <c r="K30" s="71"/>
       <c r="L30" s="2"/>
-      <c r="M30" s="57" t="s">
+      <c r="M30" s="71" t="s">
         <v>18</v>
       </c>
-      <c r="N30" s="57"/>
+      <c r="N30" s="71"/>
       <c r="O30" s="26" t="s">
         <v>55</v>
       </c>
@@ -2701,7 +3727,7 @@
       </c>
     </row>
     <row r="31" spans="4:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D31" s="69"/>
+      <c r="D31" s="81"/>
       <c r="E31" s="29" t="s">
         <v>12</v>
       </c>
@@ -2742,7 +3768,7 @@
       <c r="Q31" s="2"/>
     </row>
     <row r="32" spans="4:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D32" s="69"/>
+      <c r="D32" s="81"/>
       <c r="E32" s="29" t="s">
         <v>13</v>
       </c>
@@ -2783,7 +3809,7 @@
       <c r="Q32" s="2"/>
     </row>
     <row r="33" spans="4:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D33" s="69"/>
+      <c r="D33" s="81"/>
       <c r="E33" s="29" t="s">
         <v>14</v>
       </c>
@@ -2824,7 +3850,7 @@
       <c r="Q33" s="2"/>
     </row>
     <row r="34" spans="4:17" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D34" s="69"/>
+      <c r="D34" s="81"/>
       <c r="E34" s="2" t="s">
         <v>15</v>
       </c>
@@ -2875,7 +3901,7 @@
       </c>
     </row>
     <row r="35" spans="4:17" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D35" s="69"/>
+      <c r="D35" s="81"/>
       <c r="E35" s="2" t="s">
         <v>16</v>
       </c>
@@ -2909,43 +3935,43 @@
       <c r="Q35" s="2"/>
     </row>
     <row r="38" spans="4:17" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E38" s="57" t="s">
+      <c r="E38" s="71" t="s">
         <v>52</v>
       </c>
-      <c r="F38" s="57"/>
-      <c r="G38" s="57"/>
-      <c r="H38" s="75" t="s">
+      <c r="F38" s="71"/>
+      <c r="G38" s="71"/>
+      <c r="H38" s="83" t="s">
         <v>19</v>
       </c>
-      <c r="I38" s="76"/>
-      <c r="J38" s="76"/>
-      <c r="K38" s="76"/>
-      <c r="L38" s="76"/>
-      <c r="M38" s="76"/>
-      <c r="N38" s="76"/>
-      <c r="O38" s="76"/>
-      <c r="P38" s="76"/>
-      <c r="Q38" s="77"/>
+      <c r="I38" s="84"/>
+      <c r="J38" s="84"/>
+      <c r="K38" s="84"/>
+      <c r="L38" s="84"/>
+      <c r="M38" s="84"/>
+      <c r="N38" s="84"/>
+      <c r="O38" s="84"/>
+      <c r="P38" s="84"/>
+      <c r="Q38" s="85"/>
     </row>
     <row r="39" spans="4:17" ht="25.5" hidden="1" x14ac:dyDescent="0.2">
       <c r="E39" s="2"/>
-      <c r="F39" s="57" t="s">
+      <c r="F39" s="71" t="s">
         <v>9</v>
       </c>
-      <c r="G39" s="57"/>
-      <c r="H39" s="57" t="s">
+      <c r="G39" s="71"/>
+      <c r="H39" s="71" t="s">
         <v>43</v>
       </c>
-      <c r="I39" s="57"/>
-      <c r="J39" s="57" t="s">
+      <c r="I39" s="71"/>
+      <c r="J39" s="71" t="s">
         <v>44</v>
       </c>
-      <c r="K39" s="57"/>
+      <c r="K39" s="71"/>
       <c r="L39" s="2"/>
-      <c r="M39" s="57" t="s">
+      <c r="M39" s="71" t="s">
         <v>45</v>
       </c>
-      <c r="N39" s="57"/>
+      <c r="N39" s="71"/>
       <c r="O39" s="19" t="s">
         <v>66</v>
       </c>
@@ -3156,12 +4182,11 @@
     </row>
     <row r="50" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G50" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="50">
-    <mergeCell ref="H38:Q38"/>
     <mergeCell ref="L5:L6"/>
     <mergeCell ref="J5:J6"/>
     <mergeCell ref="J7:J8"/>
@@ -3171,8 +4196,11 @@
     <mergeCell ref="K9:K10"/>
     <mergeCell ref="L7:L8"/>
     <mergeCell ref="L9:L10"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="E12:O12"/>
+    <mergeCell ref="J13:O13"/>
+    <mergeCell ref="E13:I13"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="E29:Q29"/>
     <mergeCell ref="M39:N39"/>
     <mergeCell ref="E38:G38"/>
     <mergeCell ref="H14:I14"/>
@@ -3180,11 +4208,7 @@
     <mergeCell ref="F39:G39"/>
     <mergeCell ref="H39:I39"/>
     <mergeCell ref="J39:K39"/>
-    <mergeCell ref="E12:O12"/>
-    <mergeCell ref="J13:O13"/>
-    <mergeCell ref="E13:I13"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="E29:Q29"/>
+    <mergeCell ref="H38:Q38"/>
     <mergeCell ref="D15:D19"/>
     <mergeCell ref="F30:G30"/>
     <mergeCell ref="H30:I30"/>
@@ -3211,6 +4235,8 @@
     <mergeCell ref="G7:G8"/>
     <mergeCell ref="H7:H8"/>
     <mergeCell ref="E5:E6"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="E9:E10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3351,7 +4377,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BD7E673-853E-4343-94E1-725EDA103DB7}">
-  <dimension ref="B2:J19"/>
+  <dimension ref="B2:N44"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="20.42578125" customWidth="1"/>
@@ -3362,27 +4388,28 @@
     <col min="9" max="9" width="29" customWidth="1"/>
     <col min="10" max="10" width="36" customWidth="1"/>
     <col min="12" max="13" width="9.140625" customWidth="1"/>
+    <col min="14" max="14" width="189.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="H2" s="78" t="s">
+      <c r="H2" s="90" t="s">
         <v>71</v>
       </c>
-      <c r="I2" s="78"/>
+      <c r="I2" s="90"/>
     </row>
     <row r="3" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="H3" s="78"/>
-      <c r="I3" s="78"/>
+      <c r="H3" s="90"/>
+      <c r="I3" s="90"/>
     </row>
     <row r="4" spans="2:10" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="79" t="s">
+      <c r="B4" s="91" t="s">
         <v>72</v>
       </c>
-      <c r="C4" s="79"/>
-      <c r="D4" s="79"/>
+      <c r="C4" s="91"/>
+      <c r="D4" s="91"/>
       <c r="E4" s="7"/>
-      <c r="H4" s="78"/>
-      <c r="I4" s="78"/>
+      <c r="H4" s="90"/>
+      <c r="I4" s="90"/>
     </row>
     <row r="5" spans="2:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="34" t="s">
@@ -3395,8 +4422,8 @@
         <v>75</v>
       </c>
       <c r="E5" s="7"/>
-      <c r="H5" s="78"/>
-      <c r="I5" s="78"/>
+      <c r="H5" s="90"/>
+      <c r="I5" s="90"/>
     </row>
     <row r="6" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B6" s="37" t="s">
@@ -3410,8 +4437,8 @@
         <v>1.008</v>
       </c>
       <c r="E6" s="7"/>
-      <c r="H6" s="78"/>
-      <c r="I6" s="78"/>
+      <c r="H6" s="90"/>
+      <c r="I6" s="90"/>
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B7" s="39" t="s">
@@ -3427,14 +4454,14 @@
       <c r="E7" s="7"/>
     </row>
     <row r="8" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="H8" s="78" t="s">
+      <c r="H8" s="90" t="s">
         <v>78</v>
       </c>
-      <c r="I8" s="78"/>
+      <c r="I8" s="90"/>
     </row>
     <row r="9" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="H9" s="78"/>
-      <c r="I9" s="78"/>
+      <c r="H9" s="90"/>
+      <c r="I9" s="90"/>
     </row>
     <row r="10" spans="2:10" ht="30" x14ac:dyDescent="0.25">
       <c r="B10" s="36" t="s">
@@ -3452,8 +4479,8 @@
       <c r="F10" s="41" t="s">
         <v>83</v>
       </c>
-      <c r="H10" s="78"/>
-      <c r="I10" s="78"/>
+      <c r="H10" s="90"/>
+      <c r="I10" s="90"/>
     </row>
     <row r="11" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B11" s="37" t="s">
@@ -3473,8 +4500,8 @@
         <f>C11*D11</f>
         <v>1.1876860800000002</v>
       </c>
-      <c r="H11" s="78"/>
-      <c r="I11" s="78"/>
+      <c r="H11" s="90"/>
+      <c r="I11" s="90"/>
     </row>
     <row r="12" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B12" s="37" t="s">
@@ -3496,8 +4523,8 @@
         <v>0.38300260320000001</v>
       </c>
       <c r="G12" s="43"/>
-      <c r="H12" s="78"/>
-      <c r="I12" s="78"/>
+      <c r="H12" s="90"/>
+      <c r="I12" s="90"/>
     </row>
     <row r="13" spans="2:10" ht="30" x14ac:dyDescent="0.25">
       <c r="B13" s="44" t="s">
@@ -3530,8 +4557,8 @@
       </c>
     </row>
     <row r="15" spans="2:10" ht="42.75" x14ac:dyDescent="0.25">
-      <c r="B15" s="80"/>
-      <c r="C15" s="80"/>
+      <c r="B15" s="92"/>
+      <c r="C15" s="92"/>
       <c r="H15" s="45" t="s">
         <v>91</v>
       </c>
@@ -3555,7 +4582,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="17" spans="2:10" ht="57" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:14" ht="57" x14ac:dyDescent="0.25">
       <c r="B17" s="50"/>
       <c r="C17" s="51"/>
       <c r="H17" s="45" t="s">
@@ -3568,20 +4595,231 @@
         <v>96</v>
       </c>
     </row>
-    <row r="18" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B18" s="50"/>
       <c r="C18" s="51"/>
     </row>
-    <row r="19" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B19" s="52"/>
       <c r="C19" s="51"/>
     </row>
+    <row r="21" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="H21" s="92" t="s">
+        <v>138</v>
+      </c>
+      <c r="I21" s="92"/>
+    </row>
+    <row r="22" spans="2:14" ht="306" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H22" s="94" t="s">
+        <v>137</v>
+      </c>
+      <c r="I22" s="94"/>
+      <c r="J22" s="94"/>
+      <c r="K22" s="93"/>
+    </row>
+    <row r="23" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="H23" s="93"/>
+      <c r="I23" s="93"/>
+      <c r="J23" s="93"/>
+      <c r="K23" s="93"/>
+    </row>
+    <row r="24" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="H24" s="93"/>
+      <c r="I24" s="93"/>
+      <c r="J24" s="93"/>
+      <c r="K24" s="93"/>
+    </row>
+    <row r="25" spans="2:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H25" s="95" t="s">
+        <v>139</v>
+      </c>
+      <c r="I25" s="96"/>
+      <c r="J25" s="96"/>
+      <c r="K25" s="96"/>
+      <c r="L25" s="96"/>
+      <c r="M25" s="96"/>
+      <c r="N25" s="96"/>
+    </row>
+    <row r="26" spans="2:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H26" s="96"/>
+      <c r="I26" s="96"/>
+      <c r="J26" s="96"/>
+      <c r="K26" s="96"/>
+      <c r="L26" s="96"/>
+      <c r="M26" s="96"/>
+      <c r="N26" s="96"/>
+    </row>
+    <row r="27" spans="2:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H27" s="96"/>
+      <c r="I27" s="96"/>
+      <c r="J27" s="96"/>
+      <c r="K27" s="96"/>
+      <c r="L27" s="96"/>
+      <c r="M27" s="96"/>
+      <c r="N27" s="96"/>
+    </row>
+    <row r="28" spans="2:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H28" s="96"/>
+      <c r="I28" s="96"/>
+      <c r="J28" s="96"/>
+      <c r="K28" s="96"/>
+      <c r="L28" s="96"/>
+      <c r="M28" s="96"/>
+      <c r="N28" s="96"/>
+    </row>
+    <row r="29" spans="2:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H29" s="96"/>
+      <c r="I29" s="96"/>
+      <c r="J29" s="96"/>
+      <c r="K29" s="96"/>
+      <c r="L29" s="96"/>
+      <c r="M29" s="96"/>
+      <c r="N29" s="96"/>
+    </row>
+    <row r="30" spans="2:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H30" s="96"/>
+      <c r="I30" s="96"/>
+      <c r="J30" s="96"/>
+      <c r="K30" s="96"/>
+      <c r="L30" s="96"/>
+      <c r="M30" s="96"/>
+      <c r="N30" s="96"/>
+    </row>
+    <row r="31" spans="2:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H31" s="96"/>
+      <c r="I31" s="96"/>
+      <c r="J31" s="96"/>
+      <c r="K31" s="96"/>
+      <c r="L31" s="96"/>
+      <c r="M31" s="96"/>
+      <c r="N31" s="96"/>
+    </row>
+    <row r="32" spans="2:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H32" s="96"/>
+      <c r="I32" s="96"/>
+      <c r="J32" s="96"/>
+      <c r="K32" s="96"/>
+      <c r="L32" s="96"/>
+      <c r="M32" s="96"/>
+      <c r="N32" s="96"/>
+    </row>
+    <row r="33" spans="8:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H33" s="96"/>
+      <c r="I33" s="96"/>
+      <c r="J33" s="96"/>
+      <c r="K33" s="96"/>
+      <c r="L33" s="96"/>
+      <c r="M33" s="96"/>
+      <c r="N33" s="96"/>
+    </row>
+    <row r="34" spans="8:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H34" s="96"/>
+      <c r="I34" s="96"/>
+      <c r="J34" s="96"/>
+      <c r="K34" s="96"/>
+      <c r="L34" s="96"/>
+      <c r="M34" s="96"/>
+      <c r="N34" s="96"/>
+    </row>
+    <row r="35" spans="8:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H35" s="96"/>
+      <c r="I35" s="96"/>
+      <c r="J35" s="96"/>
+      <c r="K35" s="96"/>
+      <c r="L35" s="96"/>
+      <c r="M35" s="96"/>
+      <c r="N35" s="96"/>
+    </row>
+    <row r="36" spans="8:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H36" s="96"/>
+      <c r="I36" s="96"/>
+      <c r="J36" s="96"/>
+      <c r="K36" s="96"/>
+      <c r="L36" s="96"/>
+      <c r="M36" s="96"/>
+      <c r="N36" s="96"/>
+    </row>
+    <row r="37" spans="8:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H37" s="96"/>
+      <c r="I37" s="96"/>
+      <c r="J37" s="96"/>
+      <c r="K37" s="96"/>
+      <c r="L37" s="96"/>
+      <c r="M37" s="96"/>
+      <c r="N37" s="96"/>
+    </row>
+    <row r="38" spans="8:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H38" s="96"/>
+      <c r="I38" s="96"/>
+      <c r="J38" s="96"/>
+      <c r="K38" s="96"/>
+      <c r="L38" s="96"/>
+      <c r="M38" s="96"/>
+      <c r="N38" s="96"/>
+    </row>
+    <row r="39" spans="8:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H39" s="96"/>
+      <c r="I39" s="96"/>
+      <c r="J39" s="96"/>
+      <c r="K39" s="96"/>
+      <c r="L39" s="96"/>
+      <c r="M39" s="96"/>
+      <c r="N39" s="96"/>
+    </row>
+    <row r="40" spans="8:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H40" s="96"/>
+      <c r="I40" s="96"/>
+      <c r="J40" s="96"/>
+      <c r="K40" s="96"/>
+      <c r="L40" s="96"/>
+      <c r="M40" s="96"/>
+      <c r="N40" s="96"/>
+    </row>
+    <row r="41" spans="8:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H41" s="96"/>
+      <c r="I41" s="96"/>
+      <c r="J41" s="96"/>
+      <c r="K41" s="96"/>
+      <c r="L41" s="96"/>
+      <c r="M41" s="96"/>
+      <c r="N41" s="96"/>
+    </row>
+    <row r="42" spans="8:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H42" s="96"/>
+      <c r="I42" s="96"/>
+      <c r="J42" s="96"/>
+      <c r="K42" s="96"/>
+      <c r="L42" s="96"/>
+      <c r="M42" s="96"/>
+      <c r="N42" s="96"/>
+    </row>
+    <row r="43" spans="8:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H43" s="96"/>
+      <c r="I43" s="96"/>
+      <c r="J43" s="96"/>
+      <c r="K43" s="96"/>
+      <c r="L43" s="96"/>
+      <c r="M43" s="96"/>
+      <c r="N43" s="96"/>
+    </row>
+    <row r="44" spans="8:14" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H44" s="96"/>
+      <c r="I44" s="96"/>
+      <c r="J44" s="96"/>
+      <c r="K44" s="96"/>
+      <c r="L44" s="96"/>
+      <c r="M44" s="96"/>
+      <c r="N44" s="96"/>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="7">
+    <mergeCell ref="H25:N44"/>
     <mergeCell ref="H2:I6"/>
     <mergeCell ref="B4:D4"/>
     <mergeCell ref="H8:I12"/>
     <mergeCell ref="B15:C15"/>
+    <mergeCell ref="H22:J22"/>
+    <mergeCell ref="H21:I21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>

</xml_diff>